<commit_message>
feat(plc): update excel template with text corruption prevention rules
</commit_message>
<xml_diff>
--- a/projects/plc-monitoring-v1/GMS_자동진행_시퀀스_템플릿.xlsx
+++ b/projects/plc-monitoring-v1/GMS_자동진행_시퀀스_템플릿.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,7 +40,7 @@
     <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
-      <color rgb="001E3A8A"/>
+      <color rgb="00991B1B"/>
       <sz val="12"/>
     </font>
     <font>
@@ -57,6 +57,12 @@
       <name val="맑은 고딕"/>
       <b val="1"/>
       <color rgb="001E3A8A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
       <sz val="10"/>
     </font>
     <font>
@@ -66,7 +72,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +83,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="001E40AF"/>
         <bgColor rgb="001E40AF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEE2E2"/>
+        <bgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B91C1C"/>
+        <bgColor rgb="00B91C1C"/>
       </patternFill>
     </fill>
     <fill>
@@ -154,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -173,37 +191,41 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -571,12 +593,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -586,166 +608,171 @@
     <row r="1" ht="42" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📘 GMS 자동진행 시퀀스 엑셀 마스터 매뉴얼 &amp; 상황별 규칙 총정리</t>
+          <t>📘 GMS 자동진행 시퀀스 엑셀 마스터 매뉴얼 &amp; 표준 규칙 총정리</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>본 시트는 GMS(Gas Management System) 자동 시퀀스를 엑셀로 작성하고 수정할 때 준수해야 하는 모든 셀 규칙과 5가지 실전 상황별 예제를 담고 있습니다.</t>
+          <t>본 시트는 GMS(Gas Management System) 자동 시퀀스를 엑셀로 작성하고 수정할 때 준수해야 하는 모든 셀 규칙, 글씨 깨짐 방지 요령 및 5대 실전 예제를 담고 있습니다.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>1. 엑셀 시트 작성 3대 절대 원칙 (주의사항)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>★ [필독] 글씨 깨짐(PK... 외계어) 원인 및 올바른 파일 오픈 규칙</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>발생 원인</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>화면에 나타나는 증상</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>해결책 및 올바른 사용 방법</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>원인 1: 뷰어 오사용</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>에디터/메모장으로 열기</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>PK... docProps/app.xml 등 외계어 및 글자 깨짐 발생</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>★ .xlsx는 압축 바이너리 파일입니다. 메모장이나 VS Code 기본 텍스트 뷰어로 열지 마시고, 반드시 [Microsoft Excel], [한셀], [LibreOffice] 등 정식 스프레드시트 프로그램으로 열어야 합니다.</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>원인 2: 확장자 오류</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>.csv를 .xlsx로 강제 변경</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>서버 업로드 시 '시트를 찾을 수 없습니다' 파싱 오류</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>CSV 파일을 이름만 .xlsx로 바꾸면 안 됩니다. 반드시 엑셀에서 [다른 이름으로 저장 ➔ Excel 통합 문서(*.xlsx)]로 정식 저장하세요.</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>원인 3: 한글 인코딩</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>UTF-8 인코딩 손실</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>웹 화면에 '' 형태로 물음표 다이아몬드 깨짐</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>엑셀 내 한글 셀 내용(공정명, 메시지, 밸브명)은 표준 UTF-8 인코딩을 따르며, 저장 시 기본 통합 문서 포맷을 유지하면 100% 정상 인식됩니다.</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>1. 엑셀 시트 작성 3대 절대 원칙 (구조 규칙)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>규칙명</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>핵심 규칙 및 시스템 동작 원리</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>주의사항 (절대 금지)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>원칙 1</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>시트 이름 규칙</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>엑셀의 워크시트 이름이 시스템의 서브시퀀스 ID가 됩니다 (예: Bypass_v1, OneP_v1).</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="7" t="n"/>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>시트명을 임의로 바꾸면 시스템이 다른 시퀀스로 인식하거나 누락됩니다.</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="n"/>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>원칙 2</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>행(Row) 위치 고정</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Row 1~3은 타이틀/안내 영역, ★Row 4가 프로그램 기준 헤더 행, Row 5부터 실제 스텝 데이터입니다.</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Row 4의 열 이름을 변경하거나 헤더 위치를 위/아래로 옮기면 프로그램이 읽지 못합니다.</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>원칙 3</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>상태 유지(빈칸) 원칙</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>밸브 셀에 아무것도 적지 않은 공백(빈칸)은 '이전 스텝의 개폐 상태를 그대로 유지'함을 의미합니다.</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>매 스텝마다 모든 밸브를 O/C로 채울 필요가 없으며, 빈칸이 통신 부하와 장비 쇼크를 막습니다.</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="n"/>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>2. 실무에서 가장 많이 쓰는 5가지 상황별 엑셀 작성 예제 가이드</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>상황 구분</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>상황 명칭</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>엑셀 셀 입력 규칙 (핵심)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>상황 1</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>단순 밸브 개폐 및 안정화 대기</t>
+          <t>원칙 1</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>시트 이름 규칙</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>진행방식: 자동 / Time: 30초 / VN1: O, PNV: C, 나머지 빈칸</t>
+          <t>엑셀의 워크시트 이름이 시스템의 서브시퀀스 ID가 됩니다 (예: Bypass_v1, OneP_v1).</t>
         </is>
       </c>
       <c r="D12" s="7" t="n"/>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>공백(빈칸)은 이전 밸브 상태를 그대로 유지하므로 필요한 밸브만 O/C 입력</t>
+          <t>시트명을 임의로 바꾸면 시스템이 다른 시퀀스로 인식하거나 누락됩니다.</t>
         </is>
       </c>
       <c r="G12" s="7" t="n"/>
@@ -753,24 +780,24 @@
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>상황 2</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>진공 배기 조기통과 (Early Pass)</t>
+          <t>원칙 2</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>행(Row) 위치 고정</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Time: 120초 / Alarm Mon: VPT_{side} / 연산자: &lt;= / 설정: 0.5 / 조기통과: Y</t>
+          <t>Row 1~3은 타이틀/안내 영역, ★Row 4가 프로그램 기준 헤더 행, Row 5부터 실제 스텝 데이터입니다.</t>
         </is>
       </c>
       <c r="D13" s="7" t="n"/>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>120초가 다 지나지 않아도 0.5 Torr 도달 즉시 다음 스텝 진행 (시간 대폭 단축)</t>
+          <t>Row 4의 열 이름을 변경하거나 헤더 위치를 위/아래로 옮기면 프로그램이 읽지 못합니다.</t>
         </is>
       </c>
       <c r="G13" s="7" t="n"/>
@@ -778,888 +805,992 @@
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>상황 3</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>작업자 육안 확인 대기 (수동 ACK)</t>
+          <t>원칙 3</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>상태 유지(빈칸) 원칙</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>진행방식: 확인 / Time: 0초 / Message: '압력 확인 후 [확인] 버튼 클릭'</t>
+          <t>밸브 셀에 아무것도 적지 않은 공백(빈칸)은 '이전 스텝의 개폐 상태를 그대로 유지'함을 의미합니다.</t>
         </is>
       </c>
       <c r="D14" s="7" t="n"/>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="6" t="inlineStr">
         <is>
+          <t>매 스텝마다 모든 밸브를 O/C로 채울 필요가 없으며, 빈칸이 통신 부하와 장비 쇼크를 막습니다.</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="n"/>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>2. 실무에서 가장 많이 쓰는 5가지 상황별 엑셀 작성 예제 가이드</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>상황 구분</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>상황 명칭</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>엑셀 셀 입력 규칙 (핵심)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>상황 1</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>단순 밸브 개폐 및 안정화 대기</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>진행방식: 자동 / Time: 30초 / VN1: O, PNV: C, 나머지 빈칸</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>공백(빈칸)은 이전 밸브 상태를 그대로 유지하므로 필요한 밸브만 O/C 입력</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>상황 2</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>진공 배기 조기통과 (Early Pass)</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Time: 120초 / Alarm Mon: VPT_{side} / 연산자: &lt;= / 설정: 0.5 / 조기통과: Y</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="7" t="n"/>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>120초가 다 지나지 않아도 0.5 Torr 도달 즉시 다음 스텝 진행 (시간 대폭 단축)</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>상황 3</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>작업자 육안 확인 대기 (수동 ACK)</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>진행방식: 확인 / Time: 0초 / Message: '압력 확인 후 [확인] 버튼 클릭'</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="7" t="n"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
           <t>작업자가 HMI 화면의 확인 버튼을 누를 때까지 정지 대기 (안전 확인용)</t>
         </is>
       </c>
-      <c r="G14" s="7" t="n"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="G20" s="7" t="n"/>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>상황 4</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>밸브 순차 지연 개폐 (시차 제어)</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Time: 10초 / VN1: O (즉시 열림) / LPV_{side}: O+2 (2초 뒤 열림)</t>
         </is>
       </c>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="7" t="n"/>
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>O+n 또는 C+n 문법 사용 (용기교체 등 배관 충격 방지 순차 제어에 필수)</t>
         </is>
       </c>
-      <c r="G15" s="7" t="n"/>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="G21" s="7" t="n"/>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>상황 5</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>다회 반복 퍼지 루프 (Cycle)</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>Step 5에 Next Step: 4 / Alarm Mon: 진행횟수 / 연산자: &lt; / 설정: 3</t>
         </is>
       </c>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>진행횟수가 3회 미만이면 4번 스텝으로 루프, 3회 만족 시 6번 스텝으로 통과</t>
         </is>
       </c>
-      <c r="G16" s="7" t="n"/>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="G22" s="7" t="n"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>3. 전체 엑셀 컬럼(열)별 정밀 규칙 및 사용 방법</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>구역</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>열 헤더명</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C25" s="9" t="inlineStr">
         <is>
           <t>필수여부</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>입력 가능 값 / 문법</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>상세 설명 및 동작 방식</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>실전 입력 예시</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>S/No.</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>필수</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>1, 2, 3...</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>스텝 고유 순번입니다. 비어있는 행은 실행 시 자동으로 무시됩니다.</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>스텝 식별자</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Main Step</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>정수 (11, 20 등)</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>상위 대공정 번호입니다. 화면 상단 표시용입니다.</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>대공정</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Sub Step</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>정수 (1, 2, 3 등)</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>세부 보조 스텝 번호입니다.</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>보조 번호</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Next Step</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>스텝 번호 또는 공백</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>비워두면 다음 행으로 진행하며, 숫자를 넣으면 해당 스텝으로 무조건 점프합니다.</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>5 (또는 빈칸)</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>분기 제어</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>권장</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
         <is>
           <t>문자열</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>해당 스텝의 공정 명칭입니다. 화면 상단에 표시됩니다.</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>[ Bypass 2차 Purge ]</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>화면 표시</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Cycle</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>숫자 또는 CAPTURE:&lt;태그&gt;</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>반복 루프 표시 또는 최초 진입 시 기준 압력 캡처(P0) 지시어입니다.</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>CAPTURE:HPT_{side}</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>초기값 박제</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="9" t="inlineStr">
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>진행방식</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>필수</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>자동 / 확인 (ACK)</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>자동: 시간 경과 후 자동 진행 / 확인: 작업자가 [확인] 버튼을 누를 때까지 대기.</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>자동</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>진행 제어</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Ack Goto</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>스텝 번호 또는 공백</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>진행방식이 '확인'일 때 작업자가 버튼을 클릭하면 이동할 스텝 번호입니다.</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>확인 후 이동</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>Alarm Goto</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
         <is>
           <t>스텝 번호 또는 공백</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>이상 감지 또는 알람 발생 시 비상 조치를 위해 점프할 스텝 번호입니다.</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F34" s="5" t="inlineStr">
         <is>
           <t>99</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>알람 분기</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Message at Controller</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>문자열</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>화면 중앙 모니터 안내창에 작업자에게 띄울 안내 팝업 메시지입니다.</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F35" s="5" t="inlineStr">
         <is>
           <t>작업자 밸브 확인 요망</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>작업자 안내</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>Time (Sec)</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>필수</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D36" s="6" t="inlineStr">
         <is>
           <t>초 단위 숫자</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="E36" s="6" t="inlineStr">
         <is>
           <t>해당 스텝의 목표 유지 시간입니다. 이 시간 동안 밸브 상태를 유지합니다.</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>시간 카운트</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>고정 제어</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>Acc,Time (Sec)</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>수식 또는 숫자</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>누적 시간입니다. 보통 =SUM($K$5:K5) 수식을 넣으며 시스템이 자동 계산합니다.</t>
         </is>
       </c>
-      <c r="F31" s="5">
+      <c r="F37" s="5">
         <f>SUM($K$5:K5)</f>
         <v/>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>누적 표시</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t>밸브 태그</t>
         </is>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>밸브 태그열 (VN1 등)</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>가변</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>O, C, O+n, C+n, 공백</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>O: 열림, C: 닫힘, 공백: 이전 상태 유지, O+2: 2초 뒤 지연 열림.</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
         <is>
           <t>O (또는 O+2)</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>PLC FINS</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>감시 판정</t>
         </is>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>Alarm Monitoring</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>센서태그 / 진행횟수</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>감시할 센서명(VPT_{side}, VT) 또는 반복 횟수(진행횟수). &amp;로 다중 감시 가능.</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>VPT_{side}</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G39" s="5" t="inlineStr">
         <is>
           <t>센서 감시</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="24" customHeight="1">
-      <c r="A34" s="11" t="inlineStr">
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>감시 판정</t>
         </is>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>비교연산자</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>&lt;, &lt;=, &gt;, &gt;=, ==, ON, OFF</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>센서 현재값과 설정값을 비교할 연산자입니다. ZERO는 자동 0점 보정.</t>
         </is>
       </c>
-      <c r="F34" s="5" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t>&lt;=</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G40" s="5" t="inlineStr">
         <is>
           <t>조건 판정</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="24" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
+    <row r="41" ht="24" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
         <is>
           <t>감시 판정</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>설정명(비교대상ID)</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>CONFIG ID 또는 숫자</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>CONFIG 설정 변수명 또는 고정 수치(0.5, 3 등)를 입력합니다.</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F41" s="5" t="inlineStr">
         <is>
           <t>VAC_LIMIT 또는 0.5</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="G41" s="5" t="inlineStr">
         <is>
           <t>기준값</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="24" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
+    <row r="42" ht="24" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>감시 판정</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>조기통과</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D42" s="6" t="inlineStr">
         <is>
           <t>Y, O, 1 또는 공백</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
+      <c r="E42" s="6" t="inlineStr">
         <is>
           <t>★핵심: 시간이 다 지나지 않아도 조건 만족 시 즉시 다음 스텝으로 패스!</t>
         </is>
       </c>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="F42" s="5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G42" s="5" t="inlineStr">
         <is>
           <t>시간 단축</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="11" t="inlineStr">
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>감시 판정</t>
         </is>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>Alarm Seq.</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>1, 2, 3</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>1: 즉시 비상정지(전 밸브 Close), 2: 일시정지 후 대기, 3: 경고 배너 유지.</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F43" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G43" s="5" t="inlineStr">
         <is>
           <t>알람 동작</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>감시 판정</t>
         </is>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>Alarm Message</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D44" s="6" t="inlineStr">
         <is>
           <t>문자열</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
+      <c r="E44" s="6" t="inlineStr">
         <is>
           <t>알람 발생 시 화면에 빨간색 배너로 띄울 경고 문구입니다.</t>
         </is>
       </c>
-      <c r="F38" s="5" t="inlineStr">
+      <c r="F44" s="5" t="inlineStr">
         <is>
           <t>진공 도달 시간 초과</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="G44" s="5" t="inlineStr">
         <is>
           <t>경고 배너</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="24" customHeight="1">
-      <c r="A39" s="11" t="inlineStr">
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>감시 판정</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>선택</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>문자열</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>엔지니어 작업 메모입니다. 공정 이력 로그에 함께 기록됩니다.</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F45" s="5" t="inlineStr">
         <is>
           <t>1차 배관 진공 배기</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>엔지니어 메모</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="C16:E16"/>
+  <mergeCells count="30">
     <mergeCell ref="F11:G11"/>
-    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="C22:E22"/>
     <mergeCell ref="A4:G4"/>
-    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="D5:G5"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="A10:G10"/>
-    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F21:G21"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F17:G17"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C13:E13"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="F22:G22"/>
     <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C6:E6"/>
     <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="D7:G7"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="F14:G14"/>
+    <mergeCell ref="C20:E20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1716,17 +1847,17 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>[ 공정 제어 및 타이머 설정 구간 ]</t>
         </is>
       </c>
-      <c r="M2" s="8" t="inlineStr">
+      <c r="M2" s="10" t="inlineStr">
         <is>
           <t>[ 밸브 개폐 제어 구간 (O:열림 / C:닫힘 / 빈칸:유지) ]</t>
         </is>
       </c>
-      <c r="Z2" s="12" t="inlineStr">
+      <c r="Z2" s="14" t="inlineStr">
         <is>
           <t>[ 센서 감시 / 조기통과 / 알람 판정 구간 ]</t>
         </is>
@@ -1734,162 +1865,162 @@
     </row>
     <row r="3" ht="18" customHeight="1"/>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>S/No.</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Main Step</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Sub Step</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Next Step</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Operations</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>Cycle</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>진행방식</t>
         </is>
       </c>
-      <c r="H4" s="13" t="inlineStr">
+      <c r="H4" s="15" t="inlineStr">
         <is>
           <t>Ack Goto</t>
         </is>
       </c>
-      <c r="I4" s="13" t="inlineStr">
+      <c r="I4" s="15" t="inlineStr">
         <is>
           <t>Alarm Goto</t>
         </is>
       </c>
-      <c r="J4" s="13" t="inlineStr">
+      <c r="J4" s="15" t="inlineStr">
         <is>
           <t>Message at Controller</t>
         </is>
       </c>
-      <c r="K4" s="13" t="inlineStr">
+      <c r="K4" s="15" t="inlineStr">
         <is>
           <t>Time (Sec)</t>
         </is>
       </c>
-      <c r="L4" s="13" t="inlineStr">
+      <c r="L4" s="15" t="inlineStr">
         <is>
           <t>Acc,Time (Sec)</t>
         </is>
       </c>
-      <c r="M4" s="14" t="inlineStr">
+      <c r="M4" s="16" t="inlineStr">
         <is>
           <t>VN1</t>
         </is>
       </c>
-      <c r="N4" s="14" t="inlineStr">
+      <c r="N4" s="16" t="inlineStr">
         <is>
           <t>VN2</t>
         </is>
       </c>
-      <c r="O4" s="14" t="inlineStr">
+      <c r="O4" s="16" t="inlineStr">
         <is>
           <t>V/S_{side}</t>
         </is>
       </c>
-      <c r="P4" s="14" t="inlineStr">
+      <c r="P4" s="16" t="inlineStr">
         <is>
           <t>AG_{side}</t>
         </is>
       </c>
-      <c r="Q4" s="14" t="inlineStr">
+      <c r="Q4" s="16" t="inlineStr">
         <is>
           <t>PNV</t>
         </is>
       </c>
-      <c r="R4" s="14" t="inlineStr">
+      <c r="R4" s="16" t="inlineStr">
         <is>
           <t>GNV</t>
         </is>
       </c>
-      <c r="S4" s="14" t="inlineStr">
+      <c r="S4" s="16" t="inlineStr">
         <is>
           <t>HPIV</t>
         </is>
       </c>
-      <c r="T4" s="14" t="inlineStr">
+      <c r="T4" s="16" t="inlineStr">
         <is>
           <t>FPV_{side}</t>
         </is>
       </c>
-      <c r="U4" s="14" t="inlineStr">
+      <c r="U4" s="16" t="inlineStr">
         <is>
           <t>LPI_{side}</t>
         </is>
       </c>
-      <c r="V4" s="14" t="inlineStr">
+      <c r="V4" s="16" t="inlineStr">
         <is>
           <t>HPV_{side}</t>
         </is>
       </c>
-      <c r="W4" s="14" t="inlineStr">
+      <c r="W4" s="16" t="inlineStr">
         <is>
           <t>HPI_{side}</t>
         </is>
       </c>
-      <c r="X4" s="14" t="inlineStr">
+      <c r="X4" s="16" t="inlineStr">
         <is>
           <t>LPV_{side}</t>
         </is>
       </c>
-      <c r="Y4" s="14" t="inlineStr">
+      <c r="Y4" s="16" t="inlineStr">
         <is>
           <t>PGII_{side}</t>
         </is>
       </c>
-      <c r="Z4" s="15" t="inlineStr">
+      <c r="Z4" s="17" t="inlineStr">
         <is>
           <t>Alarm Monitoring</t>
         </is>
       </c>
-      <c r="AA4" s="15" t="inlineStr">
+      <c r="AA4" s="17" t="inlineStr">
         <is>
           <t>비교연산자</t>
         </is>
       </c>
-      <c r="AB4" s="15" t="inlineStr">
+      <c r="AB4" s="17" t="inlineStr">
         <is>
           <t>설정명(비교대상ID)</t>
         </is>
       </c>
-      <c r="AC4" s="15" t="inlineStr">
+      <c r="AC4" s="17" t="inlineStr">
         <is>
           <t>조기통과</t>
         </is>
       </c>
-      <c r="AD4" s="15" t="inlineStr">
+      <c r="AD4" s="17" t="inlineStr">
         <is>
           <t>Alarm Seq.</t>
         </is>
       </c>
-      <c r="AE4" s="15" t="inlineStr">
+      <c r="AE4" s="17" t="inlineStr">
         <is>
           <t>Alarm Message</t>
         </is>
       </c>
-      <c r="AF4" s="15" t="inlineStr">
+      <c r="AF4" s="17" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
@@ -1924,49 +2055,49 @@
           <t>Bypass 공정 시작 - 전 밸브 안전 초기화</t>
         </is>
       </c>
-      <c r="K5" s="16" t="n">
+      <c r="K5" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="L5" s="16">
+      <c r="L5" s="18">
         <f>SUM($K$5:K5)</f>
         <v/>
       </c>
-      <c r="M5" s="17" t="inlineStr">
+      <c r="M5" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="N5" s="17" t="inlineStr">
+      <c r="N5" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
       <c r="O5" s="5" t="inlineStr"/>
       <c r="P5" s="5" t="inlineStr"/>
-      <c r="Q5" s="17" t="inlineStr">
+      <c r="Q5" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="R5" s="17" t="inlineStr">
+      <c r="R5" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="S5" s="17" t="inlineStr">
+      <c r="S5" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
       <c r="T5" s="5" t="inlineStr"/>
       <c r="U5" s="5" t="inlineStr"/>
-      <c r="V5" s="17" t="inlineStr">
+      <c r="V5" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
       <c r="W5" s="5" t="inlineStr"/>
-      <c r="X5" s="17" t="inlineStr">
+      <c r="X5" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2013,14 +2144,14 @@
           <t>질소 공급 밸브 개방 (안정화 대기)</t>
         </is>
       </c>
-      <c r="K6" s="16" t="n">
+      <c r="K6" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="L6" s="16">
+      <c r="L6" s="18">
         <f>SUM($K$5:K6)</f>
         <v/>
       </c>
-      <c r="M6" s="17" t="inlineStr">
+      <c r="M6" s="19" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2028,7 +2159,7 @@
       <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr"/>
-      <c r="Q6" s="17" t="inlineStr">
+      <c r="Q6" s="19" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2084,14 +2215,14 @@
           <t>배관 진공 배기 진행 중</t>
         </is>
       </c>
-      <c r="K7" s="16" t="n">
+      <c r="K7" s="18" t="n">
         <v>120</v>
       </c>
-      <c r="L7" s="16">
+      <c r="L7" s="18">
         <f>SUM($K$5:K7)</f>
         <v/>
       </c>
-      <c r="M7" s="17" t="inlineStr">
+      <c r="M7" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2099,7 +2230,7 @@
       <c r="N7" s="5" t="inlineStr"/>
       <c r="O7" s="5" t="inlineStr"/>
       <c r="P7" s="5" t="inlineStr"/>
-      <c r="Q7" s="17" t="inlineStr">
+      <c r="Q7" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2108,7 +2239,7 @@
       <c r="S7" s="5" t="inlineStr"/>
       <c r="T7" s="5" t="inlineStr"/>
       <c r="U7" s="5" t="inlineStr"/>
-      <c r="V7" s="17" t="inlineStr">
+      <c r="V7" s="19" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2131,7 +2262,7 @@
           <t>0.5</t>
         </is>
       </c>
-      <c r="AC7" s="18" t="inlineStr">
+      <c r="AC7" s="20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -2179,10 +2310,10 @@
           <t>게이지 누설 확인 후 화면의 [확인] 버튼을 누르세요</t>
         </is>
       </c>
-      <c r="K8" s="16" t="n">
+      <c r="K8" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="16">
+      <c r="L8" s="18">
         <f>SUM($K$5:K8)</f>
         <v/>
       </c>
@@ -2240,15 +2371,15 @@
           <t>충격 방지 밸브 순차 개방 중</t>
         </is>
       </c>
-      <c r="K9" s="16" t="n">
+      <c r="K9" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="L9" s="16">
+      <c r="L9" s="18">
         <f>SUM($K$5:K9)</f>
         <v/>
       </c>
       <c r="M9" s="5" t="inlineStr"/>
-      <c r="N9" s="17" t="inlineStr">
+      <c r="N9" s="19" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2257,7 +2388,7 @@
       <c r="P9" s="5" t="inlineStr"/>
       <c r="Q9" s="5" t="inlineStr"/>
       <c r="R9" s="5" t="inlineStr"/>
-      <c r="S9" s="17" t="inlineStr">
+      <c r="S9" s="19" t="inlineStr">
         <is>
           <t>O+4</t>
         </is>
@@ -2266,7 +2397,7 @@
       <c r="U9" s="5" t="inlineStr"/>
       <c r="V9" s="5" t="inlineStr"/>
       <c r="W9" s="5" t="inlineStr"/>
-      <c r="X9" s="17" t="inlineStr">
+      <c r="X9" s="19" t="inlineStr">
         <is>
           <t>O+2</t>
         </is>
@@ -2313,14 +2444,14 @@
           <t>퍼지 가스 가압 진행</t>
         </is>
       </c>
-      <c r="K10" s="16" t="n">
+      <c r="K10" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="L10" s="16">
+      <c r="L10" s="18">
         <f>SUM($K$5:K10)</f>
         <v/>
       </c>
-      <c r="M10" s="17" t="inlineStr">
+      <c r="M10" s="19" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2328,7 +2459,7 @@
       <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr"/>
       <c r="P10" s="5" t="inlineStr"/>
-      <c r="Q10" s="17" t="inlineStr">
+      <c r="Q10" s="19" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2337,7 +2468,7 @@
       <c r="S10" s="5" t="inlineStr"/>
       <c r="T10" s="5" t="inlineStr"/>
       <c r="U10" s="5" t="inlineStr"/>
-      <c r="V10" s="17" t="inlineStr">
+      <c r="V10" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2388,14 +2519,14 @@
           <t>배기 진행 및 반복 횟수 판정</t>
         </is>
       </c>
-      <c r="K11" s="16" t="n">
+      <c r="K11" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="L11" s="16">
+      <c r="L11" s="18">
         <f>SUM($K$5:K11)</f>
         <v/>
       </c>
-      <c r="M11" s="17" t="inlineStr">
+      <c r="M11" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2403,7 +2534,7 @@
       <c r="N11" s="5" t="inlineStr"/>
       <c r="O11" s="5" t="inlineStr"/>
       <c r="P11" s="5" t="inlineStr"/>
-      <c r="Q11" s="17" t="inlineStr">
+      <c r="Q11" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2412,7 +2543,7 @@
       <c r="S11" s="5" t="inlineStr"/>
       <c r="T11" s="5" t="inlineStr"/>
       <c r="U11" s="5" t="inlineStr"/>
-      <c r="V11" s="17" t="inlineStr">
+      <c r="V11" s="19" t="inlineStr">
         <is>
           <t>O</t>
         </is>
@@ -2473,45 +2604,45 @@
           <t>Bypass 전 공정 정상 완료되었습니다</t>
         </is>
       </c>
-      <c r="K12" s="16" t="n">
+      <c r="K12" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="L12" s="16">
+      <c r="L12" s="18">
         <f>SUM($K$5:K12)</f>
         <v/>
       </c>
-      <c r="M12" s="17" t="inlineStr">
+      <c r="M12" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="N12" s="17" t="inlineStr">
+      <c r="N12" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr"/>
-      <c r="Q12" s="17" t="inlineStr">
+      <c r="Q12" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr"/>
-      <c r="S12" s="17" t="inlineStr">
+      <c r="S12" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr"/>
-      <c r="V12" s="17" t="inlineStr">
+      <c r="V12" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr"/>
-      <c r="X12" s="17" t="inlineStr">
+      <c r="X12" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2558,31 +2689,31 @@
           <t>이상 발생으로 비상 정지되었습니다. 설비를 점검하세요.</t>
         </is>
       </c>
-      <c r="K13" s="16" t="n">
+      <c r="K13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="16">
+      <c r="L13" s="18">
         <f>SUM($K$5:K13)</f>
         <v/>
       </c>
-      <c r="M13" s="17" t="inlineStr">
+      <c r="M13" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="N13" s="17" t="inlineStr">
+      <c r="N13" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
       <c r="O13" s="5" t="inlineStr"/>
       <c r="P13" s="5" t="inlineStr"/>
-      <c r="Q13" s="17" t="inlineStr">
+      <c r="Q13" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="R13" s="17" t="inlineStr">
+      <c r="R13" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
@@ -2590,13 +2721,13 @@
       <c r="S13" s="5" t="inlineStr"/>
       <c r="T13" s="5" t="inlineStr"/>
       <c r="U13" s="5" t="inlineStr"/>
-      <c r="V13" s="17" t="inlineStr">
+      <c r="V13" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
       <c r="W13" s="5" t="inlineStr"/>
-      <c r="X13" s="17" t="inlineStr">
+      <c r="X13" s="19" t="inlineStr">
         <is>
           <t>C</t>
         </is>

</xml_diff>